<commit_message>
Add new solider stat blocks for August
</commit_message>
<xml_diff>
--- a/2026_Financials.xlsx
+++ b/2026_Financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hanks\DnD-Homebrew\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6B63CD-17F7-462A-BEFA-3401B1003E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEA5856-A016-4331-BF72-4BF82D1E15B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="4" activeTab="7" xr2:uid="{A55BF991-A51A-40F9-BCC2-CFBADEB3BEC2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="4" activeTab="8" xr2:uid="{A55BF991-A51A-40F9-BCC2-CFBADEB3BEC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="226">
   <si>
     <t>Heated Desk Pad</t>
   </si>
@@ -705,6 +705,12 @@
   </si>
   <si>
     <t xml:space="preserve">Outriders </t>
+  </si>
+  <si>
+    <t>Added Extra Halerdier</t>
+  </si>
+  <si>
+    <t>Added Extra Archer &amp; Crossbowman</t>
   </si>
 </sst>
 </file>
@@ -5307,6 +5313,9 @@
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
+      <c r="J3" t="s">
+        <v>224</v>
+      </c>
       <c r="K3">
         <v>3</v>
       </c>
@@ -5314,7 +5323,7 @@
         <v>212</v>
       </c>
       <c r="M3">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
@@ -5448,6 +5457,9 @@
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
+      <c r="J7" t="s">
+        <v>225</v>
+      </c>
       <c r="K7">
         <v>2</v>
       </c>
@@ -5455,7 +5467,7 @@
         <v>213</v>
       </c>
       <c r="M7">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="N7" t="s">
         <v>215</v>
@@ -5566,7 +5578,7 @@
       </c>
       <c r="M11">
         <f>SUM(M2:M10)</f>
-        <v>234</v>
+        <v>264</v>
       </c>
       <c r="N11" t="s">
         <v>174</v>

</xml_diff>